<commit_message>
Phase 13b: fix canvas margin double-count + add faithful PNG preview renderer
Three sheets (method/planner/dashboard) prepended an extra width to canvas(),
double-counting the auto margin column and clipping labels; removed it. Add
scripts/render_preview.py (Pillow, reads real cells since soffice is broken) and
commit preview PNGs of the new premium look.
</commit_message>
<xml_diff>
--- a/asset-forge/products/P2_SK_Hospitality_Premium.xlsx
+++ b/asset-forge/products/P2_SK_Hospitality_Premium.xlsx
@@ -849,13 +849,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.4" customWidth="1" min="1" max="1"/>
-    <col width="3" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
@@ -1103,15 +1102,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I37"/>
+  <dimension ref="B1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.4" customWidth="1" min="1" max="1"/>
-    <col width="3" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
@@ -1133,10 +1131,6 @@
       <c r="C3" s="3" t="n"/>
       <c r="D3" s="3" t="n"/>
       <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="B5" s="11" t="inlineStr">
@@ -1443,17 +1437,17 @@
   </sheetData>
   <mergeCells count="14">
     <mergeCell ref="B33:D33"/>
-    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="B1:E1"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C11:E11"/>
     <mergeCell ref="B36:D36"/>
     <mergeCell ref="B37:D37"/>
     <mergeCell ref="B13:E13"/>
-    <mergeCell ref="B2:I2"/>
     <mergeCell ref="B35:D35"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="B32:E32"/>
-    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="B2:E2"/>
     <mergeCell ref="B34:D34"/>
     <mergeCell ref="C10:E10"/>
   </mergeCells>
@@ -1480,7 +1474,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.4" customWidth="1" min="1" max="1"/>
-    <col width="3" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
@@ -1491,7 +1485,6 @@
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
@@ -1517,6 +1510,9 @@
       <c r="G3" s="3" t="n"/>
       <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="n"/>
+      <c r="K3" s="3" t="n"/>
+      <c r="L3" s="3" t="n"/>
     </row>
     <row r="5" ht="4" customHeight="1">
       <c r="B5" s="23" t="inlineStr"/>
@@ -1752,12 +1748,12 @@
     <mergeCell ref="J11:L11"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="F7:H8"/>
-    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B2:L2"/>
     <mergeCell ref="B12:D13"/>
     <mergeCell ref="F12:H13"/>
-    <mergeCell ref="B1:I1"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B17:L17"/>
+    <mergeCell ref="B1:L1"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B19:L19"/>
     <mergeCell ref="F11:H11"/>

</xml_diff>

<commit_message>
Legibility guarantee: auto-fit columns + row heights so every label/header is fully readable
Samuel flagged clipped headers/labels. Add DS.fit() to design_system.py: widens
columns to fit content and grows row heights so wrapped headers show in full (only
ever increases; safe breathing-room margin). Wire it into build_pack.py (every
sheet) and build_p2_sk_premium.py. Update render_preview.py to word-wrap so PNG
previews reflect Excel. Rebuild all packs + previews.
</commit_message>
<xml_diff>
--- a/asset-forge/products/P2_SK_Hospitality_Premium.xlsx
+++ b/asset-forge/products/P2_SK_Hospitality_Premium.xlsx
@@ -845,7 +845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:K25"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.4" customWidth="1" min="1" max="1"/>
@@ -855,6 +855,10 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
@@ -881,6 +885,7 @@
       <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
         <is>
@@ -991,6 +996,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="24" customHeight="1">
       <c r="B15" s="4" t="inlineStr">
         <is>
@@ -1040,6 +1046,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="24" customHeight="1">
       <c r="B22" s="4" t="inlineStr">
         <is>
@@ -1061,6 +1068,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25" ht="22" customHeight="1">
       <c r="B25" s="10" t="inlineStr">
         <is>
@@ -1102,7 +1110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E37"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.4" customWidth="1" min="1" max="1"/>
@@ -1132,6 +1140,7 @@
       <c r="D3" s="3" t="n"/>
       <c r="E3" s="3" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5" ht="20" customHeight="1">
       <c r="B5" s="11" t="inlineStr">
         <is>
@@ -1148,6 +1157,7 @@
       </c>
       <c r="C6" s="13" t="n"/>
     </row>
+    <row r="7"/>
     <row r="8" ht="24" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
@@ -1182,6 +1192,7 @@
       </c>
       <c r="C11" s="13" t="n"/>
     </row>
+    <row r="12"/>
     <row r="13" ht="24" customHeight="1">
       <c r="B13" s="4" t="inlineStr">
         <is>
@@ -1374,6 +1385,7 @@
       <c r="D30" s="18" t="n"/>
       <c r="E30" s="18" t="n"/>
     </row>
+    <row r="31"/>
     <row r="32" ht="24" customHeight="1">
       <c r="B32" s="4" t="inlineStr">
         <is>
@@ -1470,7 +1482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:L22"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.4" customWidth="1" min="1" max="1"/>
@@ -1514,6 +1526,7 @@
       <c r="K3" s="3" t="n"/>
       <c r="L3" s="3" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5" ht="4" customHeight="1">
       <c r="B5" s="23" t="inlineStr"/>
       <c r="C5" s="24" t="n"/>
@@ -1573,6 +1586,7 @@
       <c r="K8" s="34" t="n"/>
       <c r="L8" s="35" t="n"/>
     </row>
+    <row r="9"/>
     <row r="10" ht="4" customHeight="1">
       <c r="B10" s="23" t="inlineStr"/>
       <c r="C10" s="24" t="n"/>
@@ -1632,6 +1646,7 @@
       <c r="K13" s="34" t="n"/>
       <c r="L13" s="35" t="n"/>
     </row>
+    <row r="14"/>
     <row r="15" ht="24" customHeight="1">
       <c r="B15" s="4" t="inlineStr">
         <is>
@@ -1729,6 +1744,7 @@
       <c r="K20" s="21" t="n"/>
       <c r="L20" s="21" t="n"/>
     </row>
+    <row r="21"/>
     <row r="22" ht="30" customHeight="1">
       <c r="B22" s="9" t="inlineStr">
         <is>
@@ -1787,7 +1803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O29"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.4" customWidth="1" min="1" max="1"/>
@@ -1837,6 +1853,7 @@
       <c r="N3" s="3" t="n"/>
       <c r="O3" s="3" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5" ht="20" customHeight="1">
       <c r="B5" s="11" t="inlineStr">
         <is>
@@ -2627,7 +2644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I31"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.4" customWidth="1" min="1" max="1"/>
@@ -2665,6 +2682,7 @@
       <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5" ht="20" customHeight="1">
       <c r="B5" s="11" t="inlineStr">
         <is>
@@ -3248,7 +3266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I27"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.4" customWidth="1" min="1" max="1"/>
@@ -3286,6 +3304,7 @@
       <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5" ht="20" customHeight="1">
       <c r="B5" s="11" t="inlineStr">
         <is>
@@ -3710,11 +3729,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I31"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.4" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="23.7" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
@@ -3748,6 +3767,7 @@
       <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5" ht="20" customHeight="1">
       <c r="B5" s="11" t="inlineStr">
         <is>
@@ -4132,11 +4152,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I40"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.4" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="17.1" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
@@ -4170,6 +4190,7 @@
       <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5" ht="20" customHeight="1">
       <c r="B5" s="11" t="inlineStr">
         <is>
@@ -4773,14 +4794,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:J25"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.4" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13.2" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
@@ -4813,6 +4834,7 @@
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
     </row>
+    <row r="4"/>
     <row r="5" ht="20" customHeight="1">
       <c r="B5" s="11" t="inlineStr">
         <is>
@@ -5051,6 +5073,7 @@
       <c r="I23" s="60" t="n"/>
       <c r="J23" s="53" t="n"/>
     </row>
+    <row r="24"/>
     <row r="25" ht="30" customHeight="1">
       <c r="B25" s="61" t="inlineStr">
         <is>

</xml_diff>